<commit_message>
Update ViVi PARK BD strategy and outreach assets
</commit_message>
<xml_diff>
--- a/ViVi_PARK_提案專案/00_來源資料/VIVI_案場資料庫_v1.xlsx
+++ b/ViVi_PARK_提案專案/00_來源資料/VIVI_案場資料庫_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C0378\Desktop\旺來PPT製作\ViVi_PARK_提案專案\00_來源資料\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C3F2D3-E32B-46D5-A89A-3E5F5B83D1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A08DB67A-41BB-4892-A2F7-00DEDEDF99F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14660" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Company_DD" sheetId="1" r:id="rId1"/>
@@ -2237,6 +2237,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3398,7 +3399,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>135</v>
       </c>
@@ -3469,7 +3470,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>143</v>
       </c>
@@ -3540,7 +3541,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>148</v>
       </c>
@@ -3611,7 +3612,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>151</v>
       </c>
@@ -3682,7 +3683,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>154</v>
       </c>
@@ -3753,7 +3754,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>157</v>
       </c>
@@ -3824,7 +3825,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>161</v>
       </c>
@@ -3895,7 +3896,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>164</v>
       </c>
@@ -3966,7 +3967,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>168</v>
       </c>
@@ -4037,7 +4038,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>171</v>
       </c>
@@ -4108,7 +4109,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>174</v>
       </c>
@@ -4179,7 +4180,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>179</v>
       </c>
@@ -4250,7 +4251,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>182</v>
       </c>
@@ -4321,7 +4322,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>185</v>
       </c>
@@ -4392,7 +4393,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>188</v>
       </c>
@@ -4463,7 +4464,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>191</v>
       </c>
@@ -4534,7 +4535,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>194</v>
       </c>
@@ -4605,7 +4606,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>197</v>
       </c>
@@ -4676,7 +4677,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>200</v>
       </c>
@@ -4747,7 +4748,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>205</v>
       </c>
@@ -4818,7 +4819,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>209</v>
       </c>
@@ -4889,7 +4890,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>213</v>
       </c>
@@ -4960,7 +4961,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>216</v>
       </c>
@@ -5031,7 +5032,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>219</v>
       </c>
@@ -5102,7 +5103,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>222</v>
       </c>
@@ -5173,7 +5174,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>225</v>
       </c>
@@ -5244,7 +5245,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>229</v>
       </c>
@@ -5315,7 +5316,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>232</v>
       </c>
@@ -5386,7 +5387,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>235</v>
       </c>
@@ -5457,7 +5458,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>239</v>
       </c>
@@ -5528,7 +5529,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>242</v>
       </c>
@@ -5599,7 +5600,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>245</v>
       </c>
@@ -5670,7 +5671,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>249</v>
       </c>
@@ -5741,7 +5742,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>253</v>
       </c>
@@ -5812,7 +5813,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>257</v>
       </c>
@@ -5883,7 +5884,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>260</v>
       </c>
@@ -5954,7 +5955,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>263</v>
       </c>
@@ -6025,7 +6026,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>266</v>
       </c>
@@ -6096,7 +6097,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>269</v>
       </c>
@@ -6167,7 +6168,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>272</v>
       </c>
@@ -6238,7 +6239,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>275</v>
       </c>
@@ -6309,7 +6310,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>278</v>
       </c>
@@ -6380,7 +6381,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>281</v>
       </c>
@@ -6451,7 +6452,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>284</v>
       </c>
@@ -6522,7 +6523,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>287</v>
       </c>
@@ -6593,7 +6594,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>290</v>
       </c>
@@ -6664,7 +6665,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>293</v>
       </c>
@@ -6735,7 +6736,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>296</v>
       </c>
@@ -6807,7 +6808,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W64" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:W64" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <filterColumn colId="16">
+      <filters>
+        <filter val="A"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6815,6 +6822,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7195,7 +7203,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>318</v>
       </c>
@@ -7266,7 +7274,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>322</v>
       </c>
@@ -7337,7 +7345,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>326</v>
       </c>
@@ -7834,7 +7842,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>348</v>
       </c>
@@ -7905,7 +7913,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>352</v>
       </c>
@@ -7976,7 +7984,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="29" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="29" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>356</v>
       </c>
@@ -8048,7 +8056,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W17" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:W17" xr:uid="{00000000-0009-0000-0000-000003000000}">
+    <filterColumn colId="16">
+      <filters>
+        <filter val="A"/>
+        <filter val="B+"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>